<commit_message>
Add payroll report export and continue VFP migration features.
Introduce server-side Thymeleaf/PDF/Excel export for payroll change approvals and registers, with async jobs for large batches, while extending payroll, personnel, maintenance, and frontend workflows across the Spring Boot migration.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/position-change-policy.xlsx
+++ b/docs/position-change-policy.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="174">
   <si>
     <t>职务层次</t>
   </si>
@@ -41,6 +41,15 @@
     <t>综合管理类级别范围</t>
   </si>
   <si>
+    <t>执法勤务类</t>
+  </si>
+  <si>
+    <t>执法勤务类编码</t>
+  </si>
+  <si>
+    <t>执法勤务类级别范围</t>
+  </si>
+  <si>
     <t>执法勤务警员21</t>
   </si>
   <si>
@@ -191,6 +200,12 @@
     <t>0171</t>
   </si>
   <si>
+    <t>一级警长</t>
+  </si>
+  <si>
+    <t>0201</t>
+  </si>
+  <si>
     <t>二级高级警长</t>
   </si>
   <si>
@@ -266,6 +281,12 @@
     <t>0181</t>
   </si>
   <si>
+    <t>二级警长</t>
+  </si>
+  <si>
+    <t>0202</t>
+  </si>
+  <si>
     <t>四级高级警长</t>
   </si>
   <si>
@@ -305,9 +326,6 @@
     <t>16-22</t>
   </si>
   <si>
-    <t>一级警长</t>
-  </si>
-  <si>
     <t>警务技术一级主管</t>
   </si>
   <si>
@@ -341,7 +359,10 @@
     <t>0191</t>
   </si>
   <si>
-    <t>二级警长</t>
+    <t>三级警长</t>
+  </si>
+  <si>
+    <t>0203</t>
   </si>
   <si>
     <t>警务技术二级主管</t>
@@ -380,7 +401,13 @@
     <t>17-24</t>
   </si>
   <si>
-    <t>三级警长</t>
+    <t>四级警长</t>
+  </si>
+  <si>
+    <t>0204</t>
+  </si>
+  <si>
+    <t>17-23</t>
   </si>
   <si>
     <t>警务技术三级主管</t>
@@ -407,16 +434,19 @@
     <t>三级书记员</t>
   </si>
   <si>
-    <t>17-23</t>
-  </si>
-  <si>
     <t>副科级非领导职务</t>
   </si>
   <si>
     <t>01A1</t>
   </si>
   <si>
-    <t>四级警长</t>
+    <t>一级警员</t>
+  </si>
+  <si>
+    <t>0205</t>
+  </si>
+  <si>
+    <t>18-24</t>
   </si>
   <si>
     <t>警务技术四级主管</t>
@@ -440,9 +470,6 @@
     <t>四级书记员</t>
   </si>
   <si>
-    <t>18-24</t>
-  </si>
-  <si>
     <t>科员</t>
   </si>
   <si>
@@ -452,7 +479,10 @@
     <t>18-26</t>
   </si>
   <si>
-    <t>一级警员</t>
+    <t>二级警员</t>
+  </si>
+  <si>
+    <t>0206</t>
   </si>
   <si>
     <t>警务技术员</t>
@@ -488,7 +518,10 @@
     <t>19-27</t>
   </si>
   <si>
-    <t>二级警员</t>
+    <t>三级警员</t>
+  </si>
+  <si>
+    <t>0207</t>
   </si>
   <si>
     <t>12-20</t>
@@ -510,6 +543,12 @@
   </si>
   <si>
     <t>只有从当前职务的最低级别晋升到上一职务的最低级别的，级别才有可能晋升2级，且只有科员和副科、正处和副厅，副厅和正厅的最低差2级，其他相邻职务的最低级别只差1级，也就是影响级别晋升起始年度的几乎不存在，只有从当前级别的1档晋升级别的，才会超档差，即才会影响档次晋升考核年度</t>
+  </si>
+  <si>
+    <t>职务编码前缀01到02为2010年警员套改，同职务层次套改，级别未达最低进最低，已达最低级别不变，具分析只有副科套四级警长有可能未达最低，其他都是一样的级别范围；套改到上一职务层次，级别未达最低进最低，已达最低进1级</t>
+  </si>
+  <si>
+    <t>其他类公务员到21、22警员套改，级别减7后为套改后等级，平套时，套改后等级未达最低等级的进最低等级，已达最低等级，等级不变，高套的，未达最低进最低，已达最低晋升1级；21、22回到其他类的公务员，21、22的等级+7后为其他类的级别，变动后职务层次与原职务层次相同的，级别未达变动后职务的最低级别的（这种情况不存在），进最低级别，已达最低级别的级别不变，变动后职务层次高于原职务层次的，未达最低级别，进最低级别，已达最低级别，晋升1级。</t>
   </si>
 </sst>
 </file>
@@ -1125,12 +1164,15 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1666,33 +1708,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:W16"/>
+  <dimension ref="A1:Z18"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="32" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9.54545454545454" customWidth="1"/>
     <col min="2" max="2" width="16.7272727272727" customWidth="1"/>
     <col min="3" max="4" width="20.8181818181818" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="23" customWidth="1"/>
-    <col min="7" max="8" width="18.0909090909091" customWidth="1"/>
-    <col min="9" max="9" width="29.8181818181818" customWidth="1"/>
-    <col min="10" max="10" width="16.2727272727273" customWidth="1"/>
-    <col min="11" max="11" width="9.54545454545454" customWidth="1"/>
-    <col min="12" max="12" width="16.2727272727273" customWidth="1"/>
-    <col min="13" max="13" width="9.54545454545454" customWidth="1"/>
-    <col min="14" max="14" width="18.5454545454545" customWidth="1"/>
-    <col min="15" max="15" width="5.54545454545455" customWidth="1"/>
-    <col min="16" max="16" width="18.5454545454545" customWidth="1"/>
-    <col min="17" max="17" width="5.54545454545455" customWidth="1"/>
-    <col min="18" max="18" width="20.8181818181818" customWidth="1"/>
-    <col min="19" max="19" width="5.54545454545455" customWidth="1"/>
-    <col min="20" max="20" width="16.2727272727273" customWidth="1"/>
-    <col min="21" max="21" width="5.54545454545455" customWidth="1"/>
-    <col min="22" max="22" width="16.2727272727273" customWidth="1"/>
-    <col min="23" max="23" width="8.72727272727273" style="1"/>
+    <col min="5" max="5" width="11.8181818181818" customWidth="1"/>
+    <col min="6" max="6" width="16.2727272727273" customWidth="1"/>
+    <col min="7" max="7" width="20.8181818181818" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="8.90909090909091" customWidth="1"/>
+    <col min="10" max="11" width="18.0909090909091" customWidth="1"/>
+    <col min="12" max="12" width="6.90909090909091" customWidth="1"/>
+    <col min="13" max="13" width="16.2727272727273" customWidth="1"/>
+    <col min="14" max="14" width="9.54545454545454" customWidth="1"/>
+    <col min="15" max="15" width="16.2727272727273" customWidth="1"/>
+    <col min="16" max="16" width="9.54545454545454" customWidth="1"/>
+    <col min="17" max="17" width="18.5454545454545" customWidth="1"/>
+    <col min="18" max="18" width="5.54545454545455" customWidth="1"/>
+    <col min="19" max="19" width="18.5454545454545" customWidth="1"/>
+    <col min="20" max="20" width="5.54545454545455" customWidth="1"/>
+    <col min="21" max="21" width="20.8181818181818" customWidth="1"/>
+    <col min="22" max="22" width="5.54545454545455" customWidth="1"/>
+    <col min="23" max="23" width="16.2727272727273" customWidth="1"/>
+    <col min="24" max="24" width="5.54545454545455" customWidth="1"/>
+    <col min="25" max="25" width="16.2727272727273" customWidth="1"/>
+    <col min="26" max="26" width="8.72727272727273" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:23">
+    <row r="1" customHeight="1" spans="1:26">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1730,811 +1775,883 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
       </c>
       <c r="P1" t="s">
         <v>13</v>
       </c>
-      <c r="R1" t="s">
-        <v>14</v>
-      </c>
-      <c r="T1" t="s">
+      <c r="Q1" t="s">
         <v>15</v>
       </c>
-      <c r="V1" t="s">
+      <c r="S1" t="s">
         <v>16</v>
       </c>
-      <c r="W1"/>
+      <c r="U1" t="s">
+        <v>17</v>
+      </c>
+      <c r="W1" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>19</v>
+      </c>
+      <c r="Z1"/>
     </row>
-    <row r="2" customHeight="1" spans="1:23">
+    <row r="2" customHeight="1" spans="1:26">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2">
+        <v>23</v>
+      </c>
+      <c r="H2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2">
         <v>2101</v>
       </c>
-      <c r="G2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H2">
+      <c r="J2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2">
         <v>2201</v>
       </c>
-      <c r="I2" t="s">
+      <c r="L2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N2">
+        <v>2301</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>28</v>
+      </c>
+      <c r="R2">
+        <v>2501</v>
+      </c>
+      <c r="Y2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J2" t="s">
-        <v>24</v>
-      </c>
-      <c r="K2">
-        <v>2301</v>
-      </c>
-      <c r="N2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O2">
-        <v>2501</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="W2"/>
+      <c r="Z2"/>
     </row>
-    <row r="3" customHeight="1" spans="1:23">
+    <row r="3" customHeight="1" spans="1:26">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3">
+        <v>32</v>
+      </c>
+      <c r="H3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3">
         <v>2102</v>
       </c>
-      <c r="G3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3">
+      <c r="J3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K3">
         <v>2202</v>
       </c>
-      <c r="I3" t="s">
+      <c r="L3" t="s">
+        <v>35</v>
+      </c>
+      <c r="M3" t="s">
+        <v>36</v>
+      </c>
+      <c r="N3">
+        <v>2302</v>
+      </c>
+      <c r="O3" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>38</v>
+      </c>
+      <c r="R3">
+        <v>2502</v>
+      </c>
+      <c r="S3" t="s">
+        <v>39</v>
+      </c>
+      <c r="T3">
+        <v>2602</v>
+      </c>
+      <c r="U3" t="s">
+        <v>40</v>
+      </c>
+      <c r="V3">
+        <v>2702</v>
+      </c>
+      <c r="Y3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="J3" t="s">
-        <v>33</v>
-      </c>
-      <c r="K3">
-        <v>2302</v>
-      </c>
-      <c r="L3" t="s">
-        <v>34</v>
-      </c>
-      <c r="N3" t="s">
-        <v>35</v>
-      </c>
-      <c r="O3">
-        <v>2502</v>
-      </c>
-      <c r="P3" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q3">
-        <v>2602</v>
-      </c>
-      <c r="R3" t="s">
-        <v>37</v>
-      </c>
-      <c r="S3">
-        <v>2702</v>
-      </c>
-      <c r="V3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="W3"/>
+      <c r="Z3"/>
     </row>
-    <row r="4" customHeight="1" spans="1:23">
+    <row r="4" customHeight="1" spans="1:26">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>43</v>
       </c>
       <c r="D4" t="s">
+        <v>44</v>
+      </c>
+      <c r="H4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I4">
+        <v>2103</v>
+      </c>
+      <c r="J4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K4">
+        <v>2203</v>
+      </c>
+      <c r="L4" t="s">
+        <v>47</v>
+      </c>
+      <c r="M4" t="s">
+        <v>48</v>
+      </c>
+      <c r="N4">
+        <v>2303</v>
+      </c>
+      <c r="O4" t="s">
+        <v>49</v>
+      </c>
+      <c r="P4">
+        <v>2403</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>50</v>
+      </c>
+      <c r="R4">
+        <v>2503</v>
+      </c>
+      <c r="S4" t="s">
+        <v>51</v>
+      </c>
+      <c r="T4">
+        <v>2603</v>
+      </c>
+      <c r="U4" t="s">
+        <v>52</v>
+      </c>
+      <c r="V4">
+        <v>2703</v>
+      </c>
+      <c r="W4" t="s">
+        <v>53</v>
+      </c>
+      <c r="X4">
+        <v>2803</v>
+      </c>
+      <c r="Y4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z4"/>
+    </row>
+    <row r="5" customHeight="1" spans="1:26">
+      <c r="A5" t="s">
         <v>41</v>
       </c>
-      <c r="E4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4">
-        <v>2103</v>
-      </c>
-      <c r="G4" t="s">
-        <v>43</v>
-      </c>
-      <c r="H4">
-        <v>2203</v>
-      </c>
-      <c r="I4" t="s">
+      <c r="B5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" t="s">
         <v>44</v>
       </c>
-      <c r="J4" t="s">
-        <v>45</v>
-      </c>
-      <c r="K4">
-        <v>2303</v>
-      </c>
-      <c r="L4" t="s">
-        <v>46</v>
-      </c>
-      <c r="M4">
-        <v>2403</v>
-      </c>
-      <c r="N4" t="s">
-        <v>47</v>
-      </c>
-      <c r="O4">
-        <v>2503</v>
-      </c>
-      <c r="P4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q4">
-        <v>2603</v>
-      </c>
-      <c r="R4" t="s">
-        <v>49</v>
-      </c>
-      <c r="S4">
-        <v>2703</v>
-      </c>
-      <c r="T4" t="s">
-        <v>50</v>
-      </c>
-      <c r="U4">
-        <v>2803</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="W4"/>
+      <c r="E5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H5" t="s">
+        <v>59</v>
+      </c>
+      <c r="I5">
+        <v>2104</v>
+      </c>
+      <c r="J5" t="s">
+        <v>60</v>
+      </c>
+      <c r="K5">
+        <v>2204</v>
+      </c>
+      <c r="L5" t="s">
+        <v>61</v>
+      </c>
+      <c r="M5" t="s">
+        <v>62</v>
+      </c>
+      <c r="N5">
+        <v>2304</v>
+      </c>
+      <c r="O5" t="s">
+        <v>63</v>
+      </c>
+      <c r="P5">
+        <v>2404</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>64</v>
+      </c>
+      <c r="R5">
+        <v>2504</v>
+      </c>
+      <c r="S5" t="s">
+        <v>65</v>
+      </c>
+      <c r="T5">
+        <v>2604</v>
+      </c>
+      <c r="U5" t="s">
+        <v>66</v>
+      </c>
+      <c r="V5">
+        <v>2704</v>
+      </c>
+      <c r="W5" t="s">
+        <v>67</v>
+      </c>
+      <c r="X5">
+        <v>2804</v>
+      </c>
+      <c r="Y5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z5"/>
     </row>
-    <row r="5" customHeight="1" spans="1:23">
-      <c r="A5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E5" t="s">
+    <row r="6" customHeight="1" spans="1:26">
+      <c r="A6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" t="s">
+        <v>71</v>
+      </c>
+      <c r="H6" t="s">
+        <v>72</v>
+      </c>
+      <c r="I6">
+        <v>2105</v>
+      </c>
+      <c r="J6" t="s">
+        <v>73</v>
+      </c>
+      <c r="K6">
+        <v>2205</v>
+      </c>
+      <c r="L6" t="s">
+        <v>74</v>
+      </c>
+      <c r="M6" t="s">
+        <v>75</v>
+      </c>
+      <c r="N6">
+        <v>2305</v>
+      </c>
+      <c r="O6" t="s">
+        <v>76</v>
+      </c>
+      <c r="P6">
+        <v>2405</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>77</v>
+      </c>
+      <c r="R6">
+        <v>2505</v>
+      </c>
+      <c r="S6" t="s">
+        <v>78</v>
+      </c>
+      <c r="T6">
+        <v>2605</v>
+      </c>
+      <c r="U6" t="s">
+        <v>79</v>
+      </c>
+      <c r="V6">
+        <v>2705</v>
+      </c>
+      <c r="W6" t="s">
+        <v>80</v>
+      </c>
+      <c r="X6">
+        <v>2805</v>
+      </c>
+      <c r="Y6" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="Z6"/>
+    </row>
+    <row r="7" customHeight="1" spans="1:26">
+      <c r="A7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" t="s">
+        <v>84</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="G7" t="s">
+        <v>71</v>
+      </c>
+      <c r="H7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I7">
+        <v>2106</v>
+      </c>
+      <c r="J7" t="s">
+        <v>87</v>
+      </c>
+      <c r="K7">
+        <v>2206</v>
+      </c>
+      <c r="L7" t="s">
+        <v>88</v>
+      </c>
+      <c r="M7" t="s">
+        <v>89</v>
+      </c>
+      <c r="N7">
+        <v>2306</v>
+      </c>
+      <c r="O7" t="s">
+        <v>90</v>
+      </c>
+      <c r="P7">
+        <v>2406</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>91</v>
+      </c>
+      <c r="R7">
+        <v>2506</v>
+      </c>
+      <c r="S7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T7">
+        <v>2606</v>
+      </c>
+      <c r="U7" t="s">
+        <v>93</v>
+      </c>
+      <c r="V7">
+        <v>2706</v>
+      </c>
+      <c r="W7" t="s">
+        <v>94</v>
+      </c>
+      <c r="X7">
+        <v>2806</v>
+      </c>
+      <c r="Y7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="Z7"/>
+    </row>
+    <row r="8" customHeight="1" spans="1:26">
+      <c r="A8" t="s">
+        <v>95</v>
+      </c>
+      <c r="B8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D8" t="s">
+        <v>98</v>
+      </c>
+      <c r="H8" t="s">
+        <v>57</v>
+      </c>
+      <c r="I8">
+        <v>2107</v>
+      </c>
+      <c r="J8" t="s">
+        <v>99</v>
+      </c>
+      <c r="K8">
+        <v>2207</v>
+      </c>
+      <c r="L8" t="s">
+        <v>100</v>
+      </c>
+      <c r="M8" t="s">
+        <v>101</v>
+      </c>
+      <c r="N8">
+        <v>2307</v>
+      </c>
+      <c r="O8" t="s">
+        <v>102</v>
+      </c>
+      <c r="P8">
+        <v>2407</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>103</v>
+      </c>
+      <c r="R8">
+        <v>2507</v>
+      </c>
+      <c r="S8" t="s">
+        <v>104</v>
+      </c>
+      <c r="T8">
+        <v>2607</v>
+      </c>
+      <c r="U8" t="s">
+        <v>105</v>
+      </c>
+      <c r="V8">
+        <v>2707</v>
+      </c>
+      <c r="W8" t="s">
+        <v>106</v>
+      </c>
+      <c r="X8">
+        <v>2807</v>
+      </c>
+      <c r="Y8" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="Z8"/>
+    </row>
+    <row r="9" customHeight="1" spans="1:26">
+      <c r="A9" t="s">
+        <v>95</v>
+      </c>
+      <c r="B9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="D9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E9" t="s">
+        <v>110</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="G9" t="s">
+        <v>98</v>
+      </c>
+      <c r="H9" t="s">
+        <v>84</v>
+      </c>
+      <c r="I9">
+        <v>2108</v>
+      </c>
+      <c r="J9" t="s">
+        <v>112</v>
+      </c>
+      <c r="K9">
+        <v>2208</v>
+      </c>
+      <c r="L9" t="s">
+        <v>113</v>
+      </c>
+      <c r="M9" t="s">
+        <v>114</v>
+      </c>
+      <c r="N9">
+        <v>2308</v>
+      </c>
+      <c r="O9" t="s">
+        <v>115</v>
+      </c>
+      <c r="P9">
+        <v>2408</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>116</v>
+      </c>
+      <c r="R9">
+        <v>2508</v>
+      </c>
+      <c r="S9" t="s">
+        <v>117</v>
+      </c>
+      <c r="T9">
+        <v>2608</v>
+      </c>
+      <c r="U9" t="s">
+        <v>118</v>
+      </c>
+      <c r="V9">
+        <v>2708</v>
+      </c>
+      <c r="W9" t="s">
+        <v>119</v>
+      </c>
+      <c r="X9">
+        <v>2808</v>
+      </c>
+      <c r="Y9" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="Z9"/>
+    </row>
+    <row r="10" customHeight="1" spans="1:26">
+      <c r="A10" t="s">
+        <v>120</v>
+      </c>
+      <c r="B10" t="s">
+        <v>121</v>
+      </c>
+      <c r="C10" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" t="s">
+        <v>123</v>
+      </c>
+      <c r="E10" t="s">
+        <v>124</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="G10" t="s">
+        <v>126</v>
+      </c>
+      <c r="H10" t="s">
+        <v>110</v>
+      </c>
+      <c r="I10">
+        <v>2109</v>
+      </c>
+      <c r="J10" t="s">
+        <v>127</v>
+      </c>
+      <c r="K10">
+        <v>2209</v>
+      </c>
+      <c r="L10" t="s">
+        <v>128</v>
+      </c>
+      <c r="M10" t="s">
+        <v>129</v>
+      </c>
+      <c r="N10">
+        <v>2309</v>
+      </c>
+      <c r="O10" t="s">
+        <v>130</v>
+      </c>
+      <c r="P10">
+        <v>2409</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>131</v>
+      </c>
+      <c r="R10">
+        <v>2509</v>
+      </c>
+      <c r="S10" t="s">
+        <v>132</v>
+      </c>
+      <c r="T10">
+        <v>2609</v>
+      </c>
+      <c r="U10" t="s">
+        <v>133</v>
+      </c>
+      <c r="V10">
+        <v>2709</v>
+      </c>
+      <c r="W10" t="s">
+        <v>134</v>
+      </c>
+      <c r="X10">
+        <v>2809</v>
+      </c>
+      <c r="Y10" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="Z10"/>
+    </row>
+    <row r="11" customHeight="1" spans="1:26">
+      <c r="A11" t="s">
+        <v>120</v>
+      </c>
+      <c r="B11" t="s">
+        <v>135</v>
+      </c>
+      <c r="C11" t="s">
+        <v>136</v>
+      </c>
+      <c r="D11" t="s">
+        <v>123</v>
+      </c>
+      <c r="E11" t="s">
+        <v>137</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="G11" t="s">
+        <v>139</v>
+      </c>
+      <c r="H11" t="s">
+        <v>124</v>
+      </c>
+      <c r="I11">
+        <v>2110</v>
+      </c>
+      <c r="J11" t="s">
+        <v>140</v>
+      </c>
+      <c r="K11">
+        <v>2210</v>
+      </c>
+      <c r="L11" t="s">
         <v>54</v>
       </c>
-      <c r="F5">
-        <v>2104</v>
-      </c>
-      <c r="G5" t="s">
-        <v>55</v>
-      </c>
-      <c r="H5">
-        <v>2204</v>
-      </c>
-      <c r="I5" t="s">
-        <v>56</v>
-      </c>
-      <c r="J5" t="s">
-        <v>57</v>
-      </c>
-      <c r="K5">
-        <v>2304</v>
-      </c>
-      <c r="L5" t="s">
-        <v>58</v>
-      </c>
-      <c r="M5">
-        <v>2404</v>
-      </c>
-      <c r="N5" t="s">
-        <v>59</v>
-      </c>
-      <c r="O5">
-        <v>2504</v>
-      </c>
-      <c r="P5" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q5">
-        <v>2604</v>
-      </c>
-      <c r="R5" t="s">
-        <v>61</v>
-      </c>
-      <c r="S5">
-        <v>2704</v>
-      </c>
-      <c r="T5" t="s">
-        <v>62</v>
-      </c>
-      <c r="U5">
-        <v>2804</v>
-      </c>
-      <c r="V5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="W5"/>
+      <c r="M11" t="s">
+        <v>141</v>
+      </c>
+      <c r="N11">
+        <v>2310</v>
+      </c>
+      <c r="O11" t="s">
+        <v>142</v>
+      </c>
+      <c r="P11">
+        <v>2410</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>143</v>
+      </c>
+      <c r="R11">
+        <v>2510</v>
+      </c>
+      <c r="S11" t="s">
+        <v>144</v>
+      </c>
+      <c r="T11">
+        <v>2610</v>
+      </c>
+      <c r="U11" t="s">
+        <v>145</v>
+      </c>
+      <c r="V11">
+        <v>2710</v>
+      </c>
+      <c r="W11" t="s">
+        <v>146</v>
+      </c>
+      <c r="X11">
+        <v>2810</v>
+      </c>
+      <c r="Y11" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="Z11"/>
     </row>
-    <row r="6" customHeight="1" spans="1:23">
-      <c r="A6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D6" t="s">
-        <v>66</v>
-      </c>
-      <c r="E6" t="s">
-        <v>67</v>
-      </c>
-      <c r="F6">
-        <v>2105</v>
-      </c>
-      <c r="G6" t="s">
-        <v>68</v>
-      </c>
-      <c r="H6">
-        <v>2205</v>
-      </c>
-      <c r="I6" t="s">
-        <v>69</v>
-      </c>
-      <c r="J6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K6">
-        <v>2305</v>
-      </c>
-      <c r="L6" t="s">
-        <v>71</v>
-      </c>
-      <c r="M6">
-        <v>2405</v>
-      </c>
-      <c r="N6" t="s">
-        <v>72</v>
-      </c>
-      <c r="O6">
-        <v>2505</v>
-      </c>
-      <c r="P6" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q6">
-        <v>2605</v>
-      </c>
-      <c r="R6" t="s">
-        <v>74</v>
-      </c>
-      <c r="S6">
-        <v>2705</v>
-      </c>
-      <c r="T6" t="s">
-        <v>75</v>
-      </c>
-      <c r="U6">
-        <v>2805</v>
-      </c>
-      <c r="V6" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="W6"/>
+    <row r="12" customHeight="1" spans="1:26">
+      <c r="A12" t="s">
+        <v>147</v>
+      </c>
+      <c r="B12" t="s">
+        <v>147</v>
+      </c>
+      <c r="C12" t="s">
+        <v>148</v>
+      </c>
+      <c r="D12" t="s">
+        <v>149</v>
+      </c>
+      <c r="E12" t="s">
+        <v>150</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="G12" t="s">
+        <v>149</v>
+      </c>
+      <c r="H12" t="s">
+        <v>137</v>
+      </c>
+      <c r="I12">
+        <v>2111</v>
+      </c>
+      <c r="J12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K12">
+        <v>2211</v>
+      </c>
+      <c r="L12" t="s">
+        <v>153</v>
+      </c>
+      <c r="M12" t="s">
+        <v>154</v>
+      </c>
+      <c r="N12">
+        <v>2311</v>
+      </c>
+      <c r="O12" t="s">
+        <v>155</v>
+      </c>
+      <c r="P12">
+        <v>2411</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>156</v>
+      </c>
+      <c r="R12">
+        <v>2511</v>
+      </c>
+      <c r="S12" t="s">
+        <v>157</v>
+      </c>
+      <c r="T12">
+        <v>2611</v>
+      </c>
+      <c r="U12" t="s">
+        <v>158</v>
+      </c>
+      <c r="V12">
+        <v>2711</v>
+      </c>
+      <c r="W12" t="s">
+        <v>159</v>
+      </c>
+      <c r="X12">
+        <v>2811</v>
+      </c>
+      <c r="Y12" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="Z12"/>
     </row>
-    <row r="7" customHeight="1" spans="1:23">
-      <c r="A7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B7" t="s">
-        <v>77</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="D7" t="s">
-        <v>66</v>
-      </c>
-      <c r="E7" t="s">
-        <v>79</v>
-      </c>
-      <c r="F7">
-        <v>2106</v>
-      </c>
-      <c r="G7" t="s">
-        <v>80</v>
-      </c>
-      <c r="H7">
-        <v>2206</v>
-      </c>
-      <c r="I7" t="s">
-        <v>81</v>
-      </c>
-      <c r="J7" t="s">
-        <v>82</v>
-      </c>
-      <c r="K7">
-        <v>2306</v>
-      </c>
-      <c r="L7" t="s">
-        <v>83</v>
-      </c>
-      <c r="M7">
-        <v>2406</v>
-      </c>
-      <c r="N7" t="s">
-        <v>84</v>
-      </c>
-      <c r="O7">
-        <v>2506</v>
-      </c>
-      <c r="P7" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q7">
-        <v>2606</v>
-      </c>
-      <c r="R7" t="s">
-        <v>86</v>
-      </c>
-      <c r="S7">
-        <v>2706</v>
-      </c>
-      <c r="T7" t="s">
-        <v>87</v>
-      </c>
-      <c r="U7">
-        <v>2806</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="W7"/>
+    <row r="13" customHeight="1" spans="1:26">
+      <c r="A13" t="s">
+        <v>160</v>
+      </c>
+      <c r="B13" t="s">
+        <v>160</v>
+      </c>
+      <c r="C13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D13" t="s">
+        <v>162</v>
+      </c>
+      <c r="E13" t="s">
+        <v>163</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="G13" t="s">
+        <v>162</v>
+      </c>
+      <c r="H13" t="s">
+        <v>150</v>
+      </c>
+      <c r="I13">
+        <v>2112</v>
+      </c>
+      <c r="K13">
+        <v>2212</v>
+      </c>
+      <c r="L13" t="s">
+        <v>165</v>
+      </c>
+      <c r="M13" t="s">
+        <v>166</v>
+      </c>
+      <c r="N13">
+        <v>2312</v>
+      </c>
+      <c r="O13" t="s">
+        <v>167</v>
+      </c>
+      <c r="P13">
+        <v>2412</v>
+      </c>
+      <c r="R13">
+        <v>2512</v>
+      </c>
+      <c r="T13">
+        <v>2612</v>
+      </c>
+      <c r="V13">
+        <v>2712</v>
+      </c>
+      <c r="W13" t="s">
+        <v>168</v>
+      </c>
+      <c r="X13">
+        <v>2812</v>
+      </c>
+      <c r="Y13" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="Z13"/>
     </row>
-    <row r="8" customHeight="1" spans="1:23">
-      <c r="A8" t="s">
-        <v>88</v>
-      </c>
-      <c r="B8" t="s">
-        <v>89</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="D8" t="s">
-        <v>91</v>
-      </c>
-      <c r="E8" t="s">
-        <v>92</v>
-      </c>
-      <c r="F8">
-        <v>2107</v>
-      </c>
-      <c r="G8" t="s">
-        <v>93</v>
-      </c>
-      <c r="H8">
-        <v>2207</v>
-      </c>
-      <c r="I8" t="s">
-        <v>94</v>
-      </c>
-      <c r="J8" t="s">
-        <v>95</v>
-      </c>
-      <c r="K8">
-        <v>2307</v>
-      </c>
-      <c r="L8" t="s">
-        <v>96</v>
-      </c>
-      <c r="M8">
-        <v>2407</v>
-      </c>
-      <c r="N8" t="s">
-        <v>97</v>
-      </c>
-      <c r="O8">
-        <v>2507</v>
-      </c>
-      <c r="P8" t="s">
-        <v>98</v>
-      </c>
-      <c r="Q8">
-        <v>2607</v>
-      </c>
-      <c r="R8" t="s">
-        <v>99</v>
-      </c>
-      <c r="S8">
-        <v>2707</v>
-      </c>
-      <c r="T8" t="s">
-        <v>100</v>
-      </c>
-      <c r="U8">
-        <v>2807</v>
-      </c>
-      <c r="V8" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="W8"/>
-    </row>
-    <row r="9" customHeight="1" spans="1:23">
-      <c r="A9" t="s">
-        <v>88</v>
-      </c>
-      <c r="B9" t="s">
-        <v>102</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="D9" t="s">
-        <v>91</v>
-      </c>
-      <c r="E9" t="s">
-        <v>104</v>
-      </c>
-      <c r="F9">
-        <v>2108</v>
-      </c>
-      <c r="G9" t="s">
-        <v>105</v>
-      </c>
-      <c r="H9">
-        <v>2208</v>
-      </c>
-      <c r="I9" t="s">
-        <v>106</v>
-      </c>
-      <c r="J9" t="s">
-        <v>107</v>
-      </c>
-      <c r="K9">
-        <v>2308</v>
-      </c>
-      <c r="L9" t="s">
-        <v>108</v>
-      </c>
-      <c r="M9">
-        <v>2408</v>
-      </c>
-      <c r="N9" t="s">
-        <v>109</v>
-      </c>
-      <c r="O9">
-        <v>2508</v>
-      </c>
-      <c r="P9" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q9">
-        <v>2608</v>
-      </c>
-      <c r="R9" t="s">
-        <v>111</v>
-      </c>
-      <c r="S9">
-        <v>2708</v>
-      </c>
-      <c r="T9" t="s">
-        <v>112</v>
-      </c>
-      <c r="U9">
-        <v>2808</v>
-      </c>
-      <c r="V9" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="W9"/>
-    </row>
-    <row r="10" customHeight="1" spans="1:23">
-      <c r="A10" t="s">
-        <v>113</v>
-      </c>
-      <c r="B10" t="s">
-        <v>114</v>
-      </c>
-      <c r="C10" t="s">
-        <v>115</v>
-      </c>
-      <c r="D10" t="s">
-        <v>116</v>
-      </c>
-      <c r="E10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F10">
-        <v>2109</v>
-      </c>
-      <c r="G10" t="s">
-        <v>118</v>
-      </c>
-      <c r="H10">
-        <v>2209</v>
-      </c>
-      <c r="I10" t="s">
-        <v>119</v>
-      </c>
-      <c r="J10" t="s">
-        <v>120</v>
-      </c>
-      <c r="K10">
-        <v>2309</v>
-      </c>
-      <c r="L10" t="s">
-        <v>121</v>
-      </c>
-      <c r="M10">
-        <v>2409</v>
-      </c>
-      <c r="N10" t="s">
-        <v>122</v>
-      </c>
-      <c r="O10">
-        <v>2509</v>
-      </c>
-      <c r="P10" t="s">
-        <v>123</v>
-      </c>
-      <c r="Q10">
-        <v>2609</v>
-      </c>
-      <c r="R10" t="s">
-        <v>124</v>
-      </c>
-      <c r="S10">
-        <v>2709</v>
-      </c>
-      <c r="T10" t="s">
-        <v>125</v>
-      </c>
-      <c r="U10">
-        <v>2809</v>
-      </c>
-      <c r="V10" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="W10"/>
-    </row>
-    <row r="11" customHeight="1" spans="1:23">
-      <c r="A11" t="s">
-        <v>113</v>
-      </c>
-      <c r="B11" t="s">
-        <v>127</v>
-      </c>
-      <c r="C11" t="s">
-        <v>128</v>
-      </c>
-      <c r="D11" t="s">
-        <v>116</v>
-      </c>
-      <c r="E11" t="s">
-        <v>129</v>
-      </c>
-      <c r="F11">
-        <v>2110</v>
-      </c>
-      <c r="G11" t="s">
-        <v>130</v>
-      </c>
-      <c r="H11">
-        <v>2210</v>
-      </c>
-      <c r="I11" t="s">
-        <v>51</v>
-      </c>
-      <c r="J11" t="s">
-        <v>131</v>
-      </c>
-      <c r="K11">
-        <v>2310</v>
-      </c>
-      <c r="L11" t="s">
-        <v>132</v>
-      </c>
-      <c r="M11">
-        <v>2410</v>
-      </c>
-      <c r="N11" t="s">
-        <v>133</v>
-      </c>
-      <c r="O11">
-        <v>2510</v>
-      </c>
-      <c r="P11" t="s">
-        <v>134</v>
-      </c>
-      <c r="Q11">
-        <v>2610</v>
-      </c>
-      <c r="R11" t="s">
-        <v>135</v>
-      </c>
-      <c r="S11">
-        <v>2710</v>
-      </c>
-      <c r="T11" t="s">
-        <v>136</v>
-      </c>
-      <c r="U11">
-        <v>2810</v>
-      </c>
-      <c r="V11" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="W11"/>
-    </row>
-    <row r="12" customHeight="1" spans="1:23">
-      <c r="A12" t="s">
-        <v>138</v>
-      </c>
-      <c r="B12" t="s">
-        <v>138</v>
-      </c>
-      <c r="C12" t="s">
-        <v>139</v>
-      </c>
-      <c r="D12" t="s">
-        <v>140</v>
-      </c>
-      <c r="E12" t="s">
-        <v>141</v>
-      </c>
-      <c r="F12">
-        <v>2111</v>
-      </c>
-      <c r="G12" t="s">
-        <v>142</v>
-      </c>
-      <c r="H12">
-        <v>2211</v>
-      </c>
-      <c r="I12" t="s">
-        <v>143</v>
-      </c>
-      <c r="J12" t="s">
-        <v>144</v>
-      </c>
-      <c r="K12">
-        <v>2311</v>
-      </c>
-      <c r="L12" t="s">
-        <v>145</v>
-      </c>
-      <c r="M12">
-        <v>2411</v>
-      </c>
-      <c r="N12" t="s">
-        <v>146</v>
-      </c>
-      <c r="O12">
-        <v>2511</v>
-      </c>
-      <c r="P12" t="s">
-        <v>147</v>
-      </c>
-      <c r="Q12">
-        <v>2611</v>
-      </c>
-      <c r="R12" t="s">
-        <v>148</v>
-      </c>
-      <c r="S12">
-        <v>2711</v>
-      </c>
-      <c r="T12" t="s">
-        <v>149</v>
-      </c>
-      <c r="U12">
-        <v>2811</v>
-      </c>
-      <c r="V12" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="W12"/>
-    </row>
-    <row r="13" customHeight="1" spans="1:23">
-      <c r="A13" t="s">
-        <v>150</v>
-      </c>
-      <c r="B13" t="s">
-        <v>150</v>
-      </c>
-      <c r="C13" t="s">
-        <v>151</v>
-      </c>
-      <c r="D13" t="s">
-        <v>152</v>
-      </c>
-      <c r="E13" t="s">
-        <v>153</v>
-      </c>
-      <c r="F13">
-        <v>2112</v>
-      </c>
-      <c r="H13">
-        <v>2212</v>
-      </c>
-      <c r="I13" t="s">
-        <v>154</v>
-      </c>
-      <c r="J13" t="s">
-        <v>155</v>
-      </c>
-      <c r="K13">
-        <v>2312</v>
-      </c>
-      <c r="L13" t="s">
-        <v>156</v>
-      </c>
-      <c r="M13">
-        <v>2412</v>
-      </c>
-      <c r="O13">
-        <v>2512</v>
-      </c>
-      <c r="Q13">
-        <v>2612</v>
-      </c>
-      <c r="S13">
-        <v>2712</v>
-      </c>
-      <c r="T13" t="s">
-        <v>157</v>
-      </c>
-      <c r="U13">
-        <v>2812</v>
-      </c>
-      <c r="V13" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="W13"/>
-    </row>
-    <row r="14" customHeight="1" spans="1:23">
+    <row r="14" customHeight="1" spans="1:26">
       <c r="A14" s="2" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -2558,10 +2675,13 @@
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
+      <c r="X14" s="2"/>
+      <c r="Y14" s="2"/>
+      <c r="Z14" s="2"/>
     </row>
-    <row r="15" customHeight="1" spans="1:22">
+    <row r="15" customHeight="1" spans="1:25">
       <c r="A15" s="2" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -2584,10 +2704,13 @@
       <c r="T15" s="2"/>
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
+      <c r="W15" s="2"/>
+      <c r="X15" s="2"/>
+      <c r="Y15" s="2"/>
     </row>
-    <row r="16" customHeight="1" spans="1:23">
+    <row r="16" customHeight="1" spans="1:26">
       <c r="A16" s="2" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -2610,13 +2733,47 @@
       <c r="T16" s="2"/>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
-      <c r="W16" s="3"/>
+      <c r="W16" s="2"/>
+      <c r="X16" s="2"/>
+      <c r="Y16" s="2"/>
+      <c r="Z16" s="4"/>
+    </row>
+    <row r="17" customHeight="1" spans="1:21">
+      <c r="A17" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="3"/>
+      <c r="N17" s="3"/>
+      <c r="O17" s="3"/>
+      <c r="P17" s="3"/>
+      <c r="Q17" s="3"/>
+      <c r="R17" s="3"/>
+      <c r="S17" s="3"/>
+      <c r="T17" s="3"/>
+      <c r="U17" s="3"/>
+    </row>
+    <row r="18" customHeight="1" spans="1:1">
+      <c r="A18" t="s">
+        <v>173</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A14:V14"/>
-    <mergeCell ref="A15:V15"/>
-    <mergeCell ref="A16:V16"/>
+  <mergeCells count="4">
+    <mergeCell ref="A14:Y14"/>
+    <mergeCell ref="A15:Y15"/>
+    <mergeCell ref="A16:Y16"/>
+    <mergeCell ref="A17:U17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>